<commit_message>
Support multi-sheet Excel files and polish scorecard styling
</commit_message>
<xml_diff>
--- a/sample_data/sales.xlsx
+++ b/sample_data/sales.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Regional_Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -6291,4 +6292,1830 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N31"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>order_id</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>order_date</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>product</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>gender</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>age</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>quantity</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>unit_price</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>discount</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>revenue</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>customer_rating</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>ORD-000583</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2023-01-01</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Fleece Hooded Sweatshirt</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>49</v>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3089.71</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>3089.71</v>
+      </c>
+      <c r="M2" t="n">
+        <v>967.7</v>
+      </c>
+      <c r="N2" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ORD-000057</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2023-01-02</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Gujarat</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Executive Rollerball Pen</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>49</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="n">
+        <v>879.1900000000001</v>
+      </c>
+      <c r="K3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1582.54</v>
+      </c>
+      <c r="M3" t="n">
+        <v>305.09</v>
+      </c>
+      <c r="N3" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ORD-000378</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>2023-01-02</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Ultra-wide Monitor</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>42</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="n">
+        <v>25891.55</v>
+      </c>
+      <c r="K4" t="n">
+        <v>15</v>
+      </c>
+      <c r="L4" t="n">
+        <v>22007.82</v>
+      </c>
+      <c r="M4" t="n">
+        <v>3841.15</v>
+      </c>
+      <c r="N4" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>ORD-000593</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>2023-01-02</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Magnetic Whiteboard</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>57</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3385.1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>15</v>
+      </c>
+      <c r="L5" t="n">
+        <v>5754.67</v>
+      </c>
+      <c r="M5" t="n">
+        <v>1774.33</v>
+      </c>
+      <c r="N5" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>ORD-000714</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>2023-01-03</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Ergonomic Mesh Chair</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>48</v>
+      </c>
+      <c r="I6" t="n">
+        <v>8</v>
+      </c>
+      <c r="J6" t="n">
+        <v>13454.56</v>
+      </c>
+      <c r="K6" t="n">
+        <v>10</v>
+      </c>
+      <c r="L6" t="n">
+        <v>96872.83</v>
+      </c>
+      <c r="M6" t="n">
+        <v>28233.58</v>
+      </c>
+      <c r="N6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>ORD-000736</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2023-01-03</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Executive Rollerball Pen</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>37</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>851.97</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>1703.94</v>
+      </c>
+      <c r="M7" t="n">
+        <v>447.64</v>
+      </c>
+      <c r="N7" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ORD-000779</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2023-01-03</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Ultra-wide Monitor</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>60</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="n">
+        <v>29024.96</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>87074.88</v>
+      </c>
+      <c r="M8" t="n">
+        <v>31459.58</v>
+      </c>
+      <c r="N8" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ORD-000005</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2023-01-04</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Heavy-Duty Binder</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>33</v>
+      </c>
+      <c r="I9" t="n">
+        <v>1</v>
+      </c>
+      <c r="J9" t="n">
+        <v>327.07</v>
+      </c>
+      <c r="K9" t="n">
+        <v>10</v>
+      </c>
+      <c r="L9" t="n">
+        <v>294.36</v>
+      </c>
+      <c r="M9" t="n">
+        <v>64.59</v>
+      </c>
+      <c r="N9" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>ORD-000761</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2023-01-04</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Motorized Standing Desk</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>65</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="n">
+        <v>25261.2</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>50522.4</v>
+      </c>
+      <c r="M10" t="n">
+        <v>12326.36</v>
+      </c>
+      <c r="N10" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>ORD-000177</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2023-01-05</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Executive Rollerball Pen</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H11" t="n">
+        <v>25</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
+      <c r="J11" t="n">
+        <v>885.23</v>
+      </c>
+      <c r="K11" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" t="n">
+        <v>1593.41</v>
+      </c>
+      <c r="M11" t="n">
+        <v>455.21</v>
+      </c>
+      <c r="N11" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>ORD-000627</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2023-01-05</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Heavy-Duty Binder</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H12" t="n">
+        <v>39</v>
+      </c>
+      <c r="I12" t="n">
+        <v>5</v>
+      </c>
+      <c r="J12" t="n">
+        <v>365.5</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>1827.5</v>
+      </c>
+      <c r="M12" t="n">
+        <v>688.14</v>
+      </c>
+      <c r="N12" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>ORD-000844</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2023-01-05</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Assam</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>Recycled Paper Ream</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>43</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>414.5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L13" t="n">
+        <v>393.77</v>
+      </c>
+      <c r="M13" t="n">
+        <v>71.29000000000001</v>
+      </c>
+      <c r="N13" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>ORD-000864</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>2023-01-05</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Modular Bookshelf</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H14" t="n">
+        <v>45</v>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
+        <v>8457.9</v>
+      </c>
+      <c r="K14" t="n">
+        <v>15</v>
+      </c>
+      <c r="L14" t="n">
+        <v>7189.22</v>
+      </c>
+      <c r="M14" t="n">
+        <v>1199.46</v>
+      </c>
+      <c r="N14" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ORD-000454</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>LED Desk Lamp</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H15" t="n">
+        <v>19</v>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="n">
+        <v>2165.81</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>2165.81</v>
+      </c>
+      <c r="M15" t="n">
+        <v>390.76</v>
+      </c>
+      <c r="N15" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ORD-000791</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>2023-01-06</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>Ergonomic Mesh Chair</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H16" t="n">
+        <v>18</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>12105.66</v>
+      </c>
+      <c r="K16" t="n">
+        <v>10</v>
+      </c>
+      <c r="L16" t="n">
+        <v>10895.09</v>
+      </c>
+      <c r="M16" t="n">
+        <v>3292.37</v>
+      </c>
+      <c r="N16" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ORD-000863</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2023-01-08</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Ultra-wide Monitor</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H17" t="n">
+        <v>59</v>
+      </c>
+      <c r="I17" t="n">
+        <v>2</v>
+      </c>
+      <c r="J17" t="n">
+        <v>29939.65</v>
+      </c>
+      <c r="K17" t="n">
+        <v>5</v>
+      </c>
+      <c r="L17" t="n">
+        <v>56885.33</v>
+      </c>
+      <c r="M17" t="n">
+        <v>14607.1</v>
+      </c>
+      <c r="N17" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ORD-000514</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2023-01-09</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Executive Rollerball Pen</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H18" t="n">
+        <v>62</v>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="n">
+        <v>799.39</v>
+      </c>
+      <c r="K18" t="n">
+        <v>10</v>
+      </c>
+      <c r="L18" t="n">
+        <v>719.45</v>
+      </c>
+      <c r="M18" t="n">
+        <v>86.34</v>
+      </c>
+      <c r="N18" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ORD-000099</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2023-01-10</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Punjab</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Ergonomic Mesh Chair</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H19" t="n">
+        <v>64</v>
+      </c>
+      <c r="I19" t="n">
+        <v>2</v>
+      </c>
+      <c r="J19" t="n">
+        <v>13069.34</v>
+      </c>
+      <c r="K19" t="n">
+        <v>10</v>
+      </c>
+      <c r="L19" t="n">
+        <v>23524.81</v>
+      </c>
+      <c r="M19" t="n">
+        <v>7746.99</v>
+      </c>
+      <c r="N19" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ORD-000571</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2023-01-11</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Magnetic Whiteboard</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H20" t="n">
+        <v>50</v>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="n">
+        <v>3156.07</v>
+      </c>
+      <c r="K20" t="n">
+        <v>10</v>
+      </c>
+      <c r="L20" t="n">
+        <v>2840.46</v>
+      </c>
+      <c r="M20" t="n">
+        <v>991.98</v>
+      </c>
+      <c r="N20" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ORD-000626</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2023-01-11</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Haryana</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Motorized Standing Desk</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>Non-Binary</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>27</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="n">
+        <v>23444.43</v>
+      </c>
+      <c r="K21" t="n">
+        <v>10</v>
+      </c>
+      <c r="L21" t="n">
+        <v>21099.99</v>
+      </c>
+      <c r="M21" t="n">
+        <v>2875.23</v>
+      </c>
+      <c r="N21" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ORD-000657</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2023-01-11</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Fleece Hooded Sweatshirt</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H22" t="n">
+        <v>49</v>
+      </c>
+      <c r="I22" t="n">
+        <v>2</v>
+      </c>
+      <c r="J22" t="n">
+        <v>3024.06</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5</v>
+      </c>
+      <c r="L22" t="n">
+        <v>5745.71</v>
+      </c>
+      <c r="M22" t="n">
+        <v>1876.35</v>
+      </c>
+      <c r="N22" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ORD-000852</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2023-01-12</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Karnataka</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Heavy-Duty Binder</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H23" t="n">
+        <v>33</v>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="n">
+        <v>368.84</v>
+      </c>
+      <c r="K23" t="n">
+        <v>5</v>
+      </c>
+      <c r="L23" t="n">
+        <v>350.4</v>
+      </c>
+      <c r="M23" t="n">
+        <v>43.36</v>
+      </c>
+      <c r="N23" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ORD-000063</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2023-01-13</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Slim-fit Denim Jeans</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Male</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>41</v>
+      </c>
+      <c r="I24" t="n">
+        <v>6</v>
+      </c>
+      <c r="J24" t="n">
+        <v>2999.02</v>
+      </c>
+      <c r="K24" t="n">
+        <v>15</v>
+      </c>
+      <c r="L24" t="n">
+        <v>15295</v>
+      </c>
+      <c r="M24" t="n">
+        <v>4366.19</v>
+      </c>
+      <c r="N24" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ORD-000066</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2023-01-13</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Kerala</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Heavy-Duty Binder</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H25" t="n">
+        <v>63</v>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" t="n">
+        <v>327.29</v>
+      </c>
+      <c r="K25" t="n">
+        <v>10</v>
+      </c>
+      <c r="L25" t="n">
+        <v>294.56</v>
+      </c>
+      <c r="M25" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="N25" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ORD-000536</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2023-01-13</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Telangana</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Wireless Earbuds</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H26" t="n">
+        <v>64</v>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" t="n">
+        <v>4847.08</v>
+      </c>
+      <c r="K26" t="n">
+        <v>10</v>
+      </c>
+      <c r="L26" t="n">
+        <v>4362.37</v>
+      </c>
+      <c r="M26" t="n">
+        <v>1355.42</v>
+      </c>
+      <c r="N26" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ORD-000104</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2023-01-14</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Goa</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Slim-fit Denim Jeans</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>64</v>
+      </c>
+      <c r="I27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" t="n">
+        <v>2633.36</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" t="n">
+        <v>2633.36</v>
+      </c>
+      <c r="M27" t="n">
+        <v>411.05</v>
+      </c>
+      <c r="N27" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ORD-000303</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>2023-01-14</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Rajasthan</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Clothing</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Breathable Running Shoes</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H28" t="n">
+        <v>36</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" t="n">
+        <v>4292.46</v>
+      </c>
+      <c r="K28" t="n">
+        <v>5</v>
+      </c>
+      <c r="L28" t="n">
+        <v>4077.84</v>
+      </c>
+      <c r="M28" t="n">
+        <v>1289.03</v>
+      </c>
+      <c r="N28" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ORD-000150</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2023-01-15</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Tamil Nadu</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Magnetic Whiteboard</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H29" t="n">
+        <v>49</v>
+      </c>
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" t="n">
+        <v>3327.98</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" t="n">
+        <v>3327.98</v>
+      </c>
+      <c r="M29" t="n">
+        <v>1176.42</v>
+      </c>
+      <c r="N29" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ORD-000268</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2023-01-15</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Maharashtra</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Executive Rollerball Pen</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>64</v>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" t="n">
+        <v>911.83</v>
+      </c>
+      <c r="K30" t="n">
+        <v>10</v>
+      </c>
+      <c r="L30" t="n">
+        <v>820.65</v>
+      </c>
+      <c r="M30" t="n">
+        <v>179.57</v>
+      </c>
+      <c r="N30" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ORD-000624</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>2023-01-15</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>West Bengal</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>LED Desk Lamp</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Female</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>49</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" t="n">
+        <v>2075.84</v>
+      </c>
+      <c r="K31" t="n">
+        <v>25</v>
+      </c>
+      <c r="L31" t="n">
+        <v>1556.88</v>
+      </c>
+      <c r="M31" t="n">
+        <v>494.18</v>
+      </c>
+      <c r="N31" t="n">
+        <v>5</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>